<commit_message>
Finished graphing the profiler steps
</commit_message>
<xml_diff>
--- a/PIMMS Validation work/Skyline comparison data/Skyline_all_analyte_detection_frequency.xlsx
+++ b/PIMMS Validation work/Skyline comparison data/Skyline_all_analyte_detection_frequency.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PFAS-IMplementor-for-Mass-Spectrometry--PIMMS-\PIMMS Validation work\Skyline comparison data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFE25CF-3AD2-400E-9127-5852F575A333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9773AE2-CC8B-4492-88FB-38E52924AF1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="32" activeTab="36" xr2:uid="{79560FBE-CED3-4771-A659-93F59127F910}"/>
   </bookViews>
@@ -8874,6 +8874,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21609D0F-1D77-4F49-A66E-58A7EFF8AA53}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
@@ -9662,6 +9667,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF4310F7-F432-4C06-AE6D-4EA24129CE24}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B1" t="s">

</xml_diff>